<commit_message>
feat: recordar tamaño, posición y estado de la ventana principal mediante json
</commit_message>
<xml_diff>
--- a/dist/data/Excel_Maestro.xlsx
+++ b/dist/data/Excel_Maestro.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,10 +101,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,7 +149,7 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <font>
@@ -333,8 +329,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H295" headerRowCount="1" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H295"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H299" headerRowCount="1" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H299"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Código" dataDxfId="7"/>
     <tableColumn id="2" name="Nombre" dataDxfId="6"/>
@@ -650,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H295"/>
+  <dimension ref="A1:H299"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="12.81640625" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -658,7 +654,7 @@
     <col width="19.7265625" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
     <col width="15.7265625" bestFit="1" customWidth="1" style="7" min="4" max="4"/>
     <col width="12.1796875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="16.1796875" customWidth="1" style="13" min="6" max="6"/>
+    <col width="16.1796875" customWidth="1" style="9" min="6" max="6"/>
     <col width="12.26953125" bestFit="1" customWidth="1" style="9" min="7" max="7"/>
     <col width="26.36328125" bestFit="1" customWidth="1" style="12" min="8" max="8"/>
     <col width="10.90625" customWidth="1" min="9" max="41"/>
@@ -728,7 +724,7 @@
       <c r="E2" s="8" t="n">
         <v>4934.38</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>3226.webp</t>
         </is>
@@ -764,7 +760,7 @@
       <c r="E3" s="8" t="n">
         <v>6068.15</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>3220.webp</t>
         </is>
@@ -800,7 +796,7 @@
       <c r="E4" s="8" t="n">
         <v>6095.98</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>3225.webp</t>
         </is>
@@ -836,7 +832,7 @@
       <c r="E5" s="8" t="n">
         <v>4810.96</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>3222.webp</t>
         </is>
@@ -872,7 +868,7 @@
       <c r="E6" s="8" t="n">
         <v>13475.77</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>3224.webp</t>
         </is>
@@ -908,7 +904,7 @@
       <c r="E7" s="8" t="n">
         <v>6387.59</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>3223.webp</t>
         </is>
@@ -942,9 +938,9 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>3853.85</v>
-      </c>
-      <c r="F8" t="inlineStr">
+        <v>3584.02</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>3215.webp</t>
         </is>
@@ -955,7 +951,7 @@
         </is>
       </c>
       <c r="H8" s="10" t="n">
-        <v>46213.96858372686</v>
+        <v>46230.65416479167</v>
       </c>
     </row>
     <row r="9">
@@ -980,7 +976,7 @@
       <c r="E9" s="8" t="n">
         <v>9680</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>3219.webp</t>
         </is>
@@ -1016,7 +1012,7 @@
       <c r="E10" s="8" t="n">
         <v>3968.8</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>3221.webp</t>
         </is>
@@ -1052,7 +1048,7 @@
       <c r="E11" s="8" t="n">
         <v>4554.44</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>3218.webp</t>
         </is>
@@ -1088,7 +1084,7 @@
       <c r="E12" s="8" t="n">
         <v>5642.23</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>3216.webp</t>
         </is>
@@ -1124,7 +1120,7 @@
       <c r="E13" s="8" t="n">
         <v>4617.36</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>3227.webp</t>
         </is>
@@ -1160,7 +1156,7 @@
       <c r="E14" s="8" t="n">
         <v>31787.91</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>3214.webp</t>
         </is>
@@ -1196,7 +1192,7 @@
       <c r="E15" s="8" t="n">
         <v>7812.97</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>3211.webp</t>
         </is>
@@ -1230,9 +1226,9 @@
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>5245.35</v>
-      </c>
-      <c r="F16" t="inlineStr">
+        <v>4877.51</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>3212.webp</t>
         </is>
@@ -1243,7 +1239,7 @@
         </is>
       </c>
       <c r="H16" s="10" t="n">
-        <v>46213.96858372686</v>
+        <v>46230.65416479167</v>
       </c>
     </row>
     <row r="17">
@@ -1268,7 +1264,7 @@
       <c r="E17" s="8" t="n">
         <v>2617.23</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>3213.webp</t>
         </is>
@@ -1304,7 +1300,7 @@
       <c r="E18" s="8" t="n">
         <v>1695.21</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>3228.webp</t>
         </is>
@@ -1340,7 +1336,7 @@
       <c r="E19" s="8" t="n">
         <v>2429.68</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>3229.webp</t>
         </is>
@@ -1376,7 +1372,7 @@
       <c r="E20" s="8" t="n">
         <v>2783</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>3230.webp</t>
         </is>
@@ -1412,7 +1408,7 @@
       <c r="E21" s="8" t="n">
         <v>5310.69</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>8722.webp</t>
         </is>
@@ -1448,7 +1444,7 @@
       <c r="E22" s="8" t="n">
         <v>7846.85</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>3217.webp</t>
         </is>
@@ -1484,7 +1480,7 @@
       <c r="E23" s="8" t="n">
         <v>2446.62</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>407.webp</t>
         </is>
@@ -1520,7 +1516,7 @@
       <c r="E24" s="8" t="n">
         <v>2609.97</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>3203.webp</t>
         </is>
@@ -1556,7 +1552,7 @@
       <c r="E25" s="8" t="n">
         <v>2487.76</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>3202.webp</t>
         </is>
@@ -1592,7 +1588,7 @@
       <c r="E26" s="8" t="n">
         <v>2439.36</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>3306.webp</t>
         </is>
@@ -1628,7 +1624,7 @@
       <c r="E27" s="8" t="n">
         <v>4781.92</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>3204.webp</t>
         </is>
@@ -1664,7 +1660,7 @@
       <c r="E28" s="8" t="n">
         <v>2035.22</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>3208.webp</t>
         </is>
@@ -1700,7 +1696,7 @@
       <c r="E29" s="8" t="n">
         <v>1358.83</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>3207.webp</t>
         </is>
@@ -1736,7 +1732,7 @@
       <c r="E30" s="8" t="n">
         <v>1785.96</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>3244.webp</t>
         </is>
@@ -1772,7 +1768,7 @@
       <c r="E31" s="8" t="n">
         <v>2390.96</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>1022.webp</t>
         </is>
@@ -1808,7 +1804,7 @@
       <c r="E32" s="8" t="n">
         <v>2390.96</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>1023.webp</t>
         </is>
@@ -1842,9 +1838,9 @@
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>1846.46</v>
-      </c>
-      <c r="F33" t="inlineStr">
+        <v>1860.98</v>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>3201.webp</t>
         </is>
@@ -1855,7 +1851,7 @@
         </is>
       </c>
       <c r="H33" s="10" t="n">
-        <v>46213.96858372686</v>
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="34">
@@ -1880,7 +1876,7 @@
       <c r="E34" s="8" t="n">
         <v>2117.5</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>3245.webp</t>
         </is>
@@ -1916,7 +1912,7 @@
       <c r="E35" s="8" t="n">
         <v>3916.77</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>3210.webp</t>
         </is>
@@ -1952,7 +1948,7 @@
       <c r="E36" s="8" t="n">
         <v>629.2</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>8734.webp</t>
         </is>
@@ -1985,7 +1981,7 @@
       <c r="E37" s="8" t="n">
         <v>895.4</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>8736.webp</t>
         </is>
@@ -2018,7 +2014,7 @@
       <c r="E38" s="8" t="n">
         <v>847</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>3012.webp</t>
         </is>
@@ -2051,7 +2047,7 @@
       <c r="E39" s="8" t="n">
         <v>773.1900000000001</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>3011.webp</t>
         </is>
@@ -2082,9 +2078,9 @@
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>1224.52</v>
-      </c>
-      <c r="F40" t="inlineStr">
+        <v>1193.06</v>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>3082.webp</t>
         </is>
@@ -2093,6 +2089,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H40" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="41">
@@ -2117,7 +2116,7 @@
       <c r="E41" s="8" t="n">
         <v>1569.37</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>8703.webp</t>
         </is>
@@ -2150,7 +2149,7 @@
       <c r="E42" s="8" t="n">
         <v>1225.73</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>2890.webp</t>
         </is>
@@ -2160,7 +2159,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H42" s="14" t="n">
+      <c r="H42" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -2186,7 +2185,7 @@
       <c r="E43" s="8" t="n">
         <v>11712.8</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
         <is>
           <t>3019.webp</t>
         </is>
@@ -2219,7 +2218,7 @@
       <c r="E44" s="8" t="n">
         <v>649.77</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>30.webp</t>
         </is>
@@ -2252,7 +2251,7 @@
       <c r="E45" s="8" t="n">
         <v>1124.09</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>31.webp</t>
         </is>
@@ -2285,7 +2284,7 @@
       <c r="E46" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>41.webp</t>
         </is>
@@ -2318,7 +2317,7 @@
       <c r="E47" s="8" t="n">
         <v>988.5700000000001</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>3142.webp</t>
         </is>
@@ -2351,7 +2350,7 @@
       <c r="E48" s="8" t="n">
         <v>1252.35</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>8811.webp</t>
         </is>
@@ -2384,7 +2383,7 @@
       <c r="E49" s="8" t="n">
         <v>1675.85</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>8733.webp</t>
         </is>
@@ -2401,12 +2400,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ALFAJOR GUAYMALLEN L/CH/FR CAJA</t>
+          <t>ALFAJOR GUAYMALLÉN L/CH/FR CAJA</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Guaymallén</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2417,7 +2416,7 @@
       <c r="E50" s="8" t="n">
         <v>9930.469999999999</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>61.webp</t>
         </is>
@@ -2434,12 +2433,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALFAJOR GUAYMALLEN ORO *48G </t>
+          <t xml:space="preserve">ALFAJOR GUAYMALLÉN ORO *48G </t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Guaymallén</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2450,7 +2449,7 @@
       <c r="E51" s="8" t="n">
         <v>522.72</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
         <is>
           <t>63.webp</t>
         </is>
@@ -2483,7 +2482,7 @@
       <c r="E52" s="8" t="n">
         <v>986.15</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>3096.webp</t>
         </is>
@@ -2493,7 +2492,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H52" s="14" t="n">
+      <c r="H52" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -2519,7 +2518,7 @@
       <c r="E53" s="8" t="n">
         <v>848.21</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>3010.webp</t>
         </is>
@@ -2552,7 +2551,7 @@
       <c r="E54" s="8" t="n">
         <v>792.55</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>2464.webp</t>
         </is>
@@ -2585,7 +2584,7 @@
       <c r="E55" s="8" t="n">
         <v>1280.18</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>3193.webp</t>
         </is>
@@ -2618,7 +2617,7 @@
       <c r="E56" s="8" t="n">
         <v>1356.41</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>8812.webp</t>
         </is>
@@ -2651,7 +2650,7 @@
       <c r="E57" s="8" t="n">
         <v>1684.32</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>3160.webp</t>
         </is>
@@ -2685,9 +2684,9 @@
         </is>
       </c>
       <c r="E58" s="8" t="n">
-        <v>1195.48</v>
-      </c>
-      <c r="F58" t="inlineStr">
+        <v>1203.95</v>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>2302.webp</t>
         </is>
@@ -2696,6 +2695,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="59">
@@ -2720,7 +2722,7 @@
       <c r="E59" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
         <is>
           <t>64.webp</t>
         </is>
@@ -2753,7 +2755,7 @@
       <c r="E60" s="8" t="n">
         <v>1225.73</v>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>50.webp</t>
         </is>
@@ -2786,7 +2788,7 @@
       <c r="E61" s="8" t="n">
         <v>7332.6</v>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>1791.webp</t>
         </is>
@@ -2819,7 +2821,7 @@
       <c r="E62" s="8" t="n">
         <v>1189.43</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>8819.webp</t>
         </is>
@@ -2852,7 +2854,7 @@
       <c r="E63" s="8" t="n">
         <v>296.45</v>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="7" t="inlineStr">
         <is>
           <t>112.webp</t>
         </is>
@@ -2885,7 +2887,7 @@
       <c r="E64" s="8" t="n">
         <v>1541.54</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>110.webp</t>
         </is>
@@ -2918,7 +2920,7 @@
       <c r="E65" s="8" t="n">
         <v>511.83</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="7" t="inlineStr">
         <is>
           <t>111.webp</t>
         </is>
@@ -2951,7 +2953,7 @@
       <c r="E66" s="8" t="n">
         <v>4388.67</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>887.webp</t>
         </is>
@@ -2961,7 +2963,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H66" s="14" t="n">
+      <c r="H66" s="10" t="n">
         <v>46226.92162092592</v>
       </c>
     </row>
@@ -2987,7 +2989,7 @@
       <c r="E67" s="8" t="n">
         <v>4750.46</v>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="7" t="inlineStr">
         <is>
           <t>3075.webp</t>
         </is>
@@ -2997,7 +2999,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H67" s="14" t="n">
+      <c r="H67" s="10" t="n">
         <v>46226.92162092592</v>
       </c>
     </row>
@@ -3023,7 +3025,7 @@
       <c r="E68" s="8" t="n">
         <v>7619.37</v>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>201.webp</t>
         </is>
@@ -3056,7 +3058,7 @@
       <c r="E69" s="8" t="n">
         <v>13519.33</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="7" t="inlineStr">
         <is>
           <t>199.webp</t>
         </is>
@@ -3089,7 +3091,7 @@
       <c r="E70" s="8" t="n">
         <v>2533.74</v>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>200.webp</t>
         </is>
@@ -3122,7 +3124,7 @@
       <c r="E71" s="8" t="n">
         <v>4485.47</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="7" t="inlineStr">
         <is>
           <t>2570.webp</t>
         </is>
@@ -3155,7 +3157,7 @@
       <c r="E72" s="8" t="n">
         <v>22748</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr">
         <is>
           <t>3055.webp</t>
         </is>
@@ -3191,7 +3193,7 @@
       <c r="E73" s="8" t="n">
         <v>16999</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>3176.webp</t>
         </is>
@@ -3222,9 +3224,9 @@
         </is>
       </c>
       <c r="E74" s="8" t="n">
-        <v>4351.16</v>
-      </c>
-      <c r="F74" t="inlineStr">
+        <v>4241.05</v>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
         <is>
           <t>335.webp</t>
         </is>
@@ -3233,6 +3235,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H74" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="75">
@@ -3257,7 +3262,7 @@
       <c r="E75" s="8" t="n">
         <v>1770.23</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="7" t="inlineStr">
         <is>
           <t>334.webp</t>
         </is>
@@ -3290,7 +3295,7 @@
       <c r="E76" s="8" t="n">
         <v>2722.5</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="7" t="inlineStr">
         <is>
           <t>339.webp</t>
         </is>
@@ -3300,7 +3305,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H76" s="14" t="n">
+      <c r="H76" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -3326,7 +3331,7 @@
       <c r="E77" s="8" t="n">
         <v>3509</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="7" t="inlineStr">
         <is>
           <t>342.webp</t>
         </is>
@@ -3359,7 +3364,7 @@
       <c r="E78" s="8" t="n">
         <v>5989.5</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="7" t="inlineStr">
         <is>
           <t>340.webp</t>
         </is>
@@ -3369,7 +3374,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H78" s="14" t="n">
+      <c r="H78" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -3395,7 +3400,7 @@
       <c r="E79" s="8" t="n">
         <v>1427.8</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="7" t="inlineStr">
         <is>
           <t>341.webp</t>
         </is>
@@ -3426,9 +3431,9 @@
         </is>
       </c>
       <c r="E80" s="8" t="n">
-        <v>2116.29</v>
-      </c>
-      <c r="F80" t="inlineStr">
+        <v>2081.2</v>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
         <is>
           <t>3084.webp</t>
         </is>
@@ -3437,6 +3442,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H80" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="81">
@@ -3461,7 +3469,7 @@
       <c r="E81" s="8" t="n">
         <v>1414.49</v>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F81" s="7" t="inlineStr">
         <is>
           <t>360.webp</t>
         </is>
@@ -3494,7 +3502,7 @@
       <c r="E82" s="8" t="n">
         <v>2282.06</v>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="7" t="inlineStr">
         <is>
           <t>6086.webp</t>
         </is>
@@ -3527,7 +3535,7 @@
       <c r="E83" s="8" t="n">
         <v>982.52</v>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F83" s="7" t="inlineStr">
         <is>
           <t>540.webp</t>
         </is>
@@ -3560,7 +3568,7 @@
       <c r="E84" s="8" t="n">
         <v>3314.19</v>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" s="7" t="inlineStr">
         <is>
           <t>3231.webp</t>
         </is>
@@ -3593,7 +3601,7 @@
       <c r="E85" s="8" t="n">
         <v>698.17</v>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="7" t="inlineStr">
         <is>
           <t>8825.webp</t>
         </is>
@@ -3626,7 +3634,7 @@
       <c r="E86" s="8" t="n">
         <v>7562.5</v>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="7" t="inlineStr">
         <is>
           <t>8806.webp</t>
         </is>
@@ -3659,7 +3667,7 @@
       <c r="E87" s="8" t="n">
         <v>2722.5</v>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="7" t="inlineStr">
         <is>
           <t>2160.webp</t>
         </is>
@@ -3692,7 +3700,7 @@
       <c r="E88" s="8" t="n">
         <v>8681.75</v>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="7" t="inlineStr">
         <is>
           <t>3056.webp</t>
         </is>
@@ -3725,7 +3733,7 @@
       <c r="E89" s="8" t="n">
         <v>718.74</v>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" s="7" t="inlineStr">
         <is>
           <t>8826.webp</t>
         </is>
@@ -3756,9 +3764,9 @@
         </is>
       </c>
       <c r="E90" s="8" t="n">
-        <v>1461.2</v>
-      </c>
-      <c r="F90" t="inlineStr">
+        <v>1697.63</v>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
         <is>
           <t>724.webp</t>
         </is>
@@ -3767,6 +3775,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H90" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="91">
@@ -3789,9 +3800,9 @@
         </is>
       </c>
       <c r="E91" s="8" t="n">
-        <v>1428.83</v>
-      </c>
-      <c r="F91" t="inlineStr">
+        <v>1697.63</v>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
         <is>
           <t>730.webp</t>
         </is>
@@ -3800,6 +3811,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H91" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="92">
@@ -3824,7 +3838,7 @@
       <c r="E92" s="8" t="n">
         <v>7593.96</v>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F92" s="7" t="inlineStr">
         <is>
           <t>3235.webp</t>
         </is>
@@ -3860,7 +3874,7 @@
       <c r="E93" s="8" t="n">
         <v>2433.31</v>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F93" s="7" t="inlineStr">
         <is>
           <t>3233.webp</t>
         </is>
@@ -3893,7 +3907,7 @@
       <c r="E94" s="8" t="n">
         <v>6558.2</v>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F94" s="7" t="inlineStr">
         <is>
           <t>3234.webp</t>
         </is>
@@ -3929,7 +3943,7 @@
       <c r="E95" s="8" t="n">
         <v>18857.85</v>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F95" s="7" t="inlineStr">
         <is>
           <t>946.webp</t>
         </is>
@@ -3962,7 +3976,7 @@
       <c r="E96" s="8" t="n">
         <v>2554.31</v>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="F96" s="7" t="inlineStr">
         <is>
           <t>949.webp</t>
         </is>
@@ -3995,7 +4009,7 @@
       <c r="E97" s="8" t="n">
         <v>2311.1</v>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
         <is>
           <t>950.webp</t>
         </is>
@@ -4028,7 +4042,7 @@
       <c r="E98" s="8" t="n">
         <v>13054.69</v>
       </c>
-      <c r="F98" t="inlineStr">
+      <c r="F98" s="7" t="inlineStr">
         <is>
           <t>954.webp</t>
         </is>
@@ -4038,7 +4052,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H98" s="14" t="n">
+      <c r="H98" s="10" t="n">
         <v>46226.92162092592</v>
       </c>
     </row>
@@ -4064,7 +4078,7 @@
       <c r="E99" s="8" t="n">
         <v>1391.5</v>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F99" s="7" t="inlineStr">
         <is>
           <t>955.webp</t>
         </is>
@@ -4097,7 +4111,7 @@
       <c r="E100" s="8" t="n">
         <v>1702.47</v>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F100" s="7" t="inlineStr">
         <is>
           <t>2745.webp</t>
         </is>
@@ -4130,7 +4144,7 @@
       <c r="E101" s="8" t="n">
         <v>6289.58</v>
       </c>
-      <c r="F101" t="inlineStr">
+      <c r="F101" s="7" t="inlineStr">
         <is>
           <t>8817.webp</t>
         </is>
@@ -4163,7 +4177,7 @@
       <c r="E102" s="8" t="n">
         <v>2821.72</v>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" s="7" t="inlineStr">
         <is>
           <t>3014.webp</t>
         </is>
@@ -4199,7 +4213,7 @@
       <c r="E103" s="8" t="n">
         <v>2807.2</v>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" s="7" t="inlineStr">
         <is>
           <t>8818.webp</t>
         </is>
@@ -4232,7 +4246,7 @@
       <c r="E104" s="8" t="n">
         <v>1274.13</v>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F104" s="7" t="inlineStr">
         <is>
           <t>3063.webp</t>
         </is>
@@ -4263,9 +4277,9 @@
         </is>
       </c>
       <c r="E105" s="8" t="n">
-        <v>3914.35</v>
-      </c>
-      <c r="F105" t="inlineStr">
+        <v>5326.42</v>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
         <is>
           <t>3018.webp</t>
         </is>
@@ -4274,6 +4288,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H105" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="106">
@@ -4298,7 +4315,7 @@
       <c r="E106" s="8" t="n">
         <v>949.85</v>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="F106" s="7" t="inlineStr">
         <is>
           <t>1220.webp</t>
         </is>
@@ -4331,7 +4348,7 @@
       <c r="E107" s="8" t="n">
         <v>733.26</v>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F107" s="7" t="inlineStr">
         <is>
           <t>1226.webp</t>
         </is>
@@ -4364,7 +4381,7 @@
       <c r="E108" s="8" t="n">
         <v>5563.58</v>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F108" s="7" t="inlineStr">
         <is>
           <t>1240.webp</t>
         </is>
@@ -4397,7 +4414,7 @@
       <c r="E109" s="8" t="n">
         <v>5336.1</v>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F109" s="7" t="inlineStr">
         <is>
           <t>8804.webp</t>
         </is>
@@ -4430,7 +4447,7 @@
       <c r="E110" s="8" t="n">
         <v>5336.1</v>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F110" s="7" t="inlineStr">
         <is>
           <t>2894.webp</t>
         </is>
@@ -4463,7 +4480,7 @@
       <c r="E111" s="8" t="n">
         <v>5563.58</v>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F111" s="7" t="inlineStr">
         <is>
           <t>1245.webp</t>
         </is>
@@ -4496,7 +4513,7 @@
       <c r="E112" s="8" t="n">
         <v>3777.62</v>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F112" s="7" t="inlineStr">
         <is>
           <t>3240.webp</t>
         </is>
@@ -4532,7 +4549,7 @@
       <c r="E113" s="8" t="n">
         <v>6893.37</v>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F113" s="7" t="inlineStr">
         <is>
           <t>3238.webp</t>
         </is>
@@ -4565,7 +4582,7 @@
       <c r="E114" s="8" t="n">
         <v>3394.05</v>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F114" s="7" t="inlineStr">
         <is>
           <t>3237.webp</t>
         </is>
@@ -4598,7 +4615,7 @@
       <c r="E115" s="8" t="n">
         <v>5585.36</v>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F115" s="7" t="inlineStr">
         <is>
           <t>3236.webp</t>
         </is>
@@ -4631,7 +4648,7 @@
       <c r="E116" s="8" t="n">
         <v>1076.9</v>
       </c>
-      <c r="F116" t="inlineStr">
+      <c r="F116" s="7" t="inlineStr">
         <is>
           <t>38.webp</t>
         </is>
@@ -4664,7 +4681,7 @@
       <c r="E117" s="8" t="n">
         <v>750.2</v>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F117" s="7" t="inlineStr">
         <is>
           <t>727.webp</t>
         </is>
@@ -4697,7 +4714,7 @@
       <c r="E118" s="8" t="n">
         <v>1007.93</v>
       </c>
-      <c r="F118" t="inlineStr">
+      <c r="F118" s="7" t="inlineStr">
         <is>
           <t>1719.webp</t>
         </is>
@@ -4730,7 +4747,7 @@
       <c r="E119" s="8" t="n">
         <v>3590.07</v>
       </c>
-      <c r="F119" t="inlineStr">
+      <c r="F119" s="7" t="inlineStr">
         <is>
           <t>3242.webp</t>
         </is>
@@ -4766,7 +4783,7 @@
       <c r="E120" s="8" t="n">
         <v>1890.02</v>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F120" s="7" t="inlineStr">
         <is>
           <t>3243.webp</t>
         </is>
@@ -4802,7 +4819,7 @@
       <c r="E121" s="8" t="n">
         <v>2203.41</v>
       </c>
-      <c r="F121" t="inlineStr">
+      <c r="F121" s="7" t="inlineStr">
         <is>
           <t>3241.webp</t>
         </is>
@@ -4838,7 +4855,7 @@
       <c r="E122" s="8" t="n">
         <v>1228.15</v>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="F122" s="7" t="inlineStr">
         <is>
           <t>1826.webp</t>
         </is>
@@ -4871,7 +4888,7 @@
       <c r="E123" s="8" t="n">
         <v>3499.32</v>
       </c>
-      <c r="F123" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr">
         <is>
           <t>1823.webp</t>
         </is>
@@ -4904,7 +4921,7 @@
       <c r="E124" s="8" t="n">
         <v>5590.2</v>
       </c>
-      <c r="F124" t="inlineStr">
+      <c r="F124" s="7" t="inlineStr">
         <is>
           <t>1825.webp</t>
         </is>
@@ -4937,7 +4954,7 @@
       <c r="E125" s="8" t="n">
         <v>4779.5</v>
       </c>
-      <c r="F125" t="inlineStr">
+      <c r="F125" s="7" t="inlineStr">
         <is>
           <t>3239.webp</t>
         </is>
@@ -4970,7 +4987,7 @@
       <c r="E126" s="8" t="n">
         <v>4176.92</v>
       </c>
-      <c r="F126" t="inlineStr">
+      <c r="F126" s="7" t="inlineStr">
         <is>
           <t>1884.webp</t>
         </is>
@@ -5003,7 +5020,7 @@
       <c r="E127" s="8" t="n">
         <v>5299.8</v>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F127" s="7" t="inlineStr">
         <is>
           <t>1885.webp</t>
         </is>
@@ -5036,7 +5053,7 @@
       <c r="E128" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F128" t="inlineStr">
+      <c r="F128" s="7" t="inlineStr">
         <is>
           <t>6075.webp</t>
         </is>
@@ -5046,7 +5063,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H128" s="14" t="n">
+      <c r="H128" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -5072,7 +5089,7 @@
       <c r="E129" s="8" t="n">
         <v>1287.44</v>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F129" s="7" t="inlineStr">
         <is>
           <t>3192.webp</t>
         </is>
@@ -5105,7 +5122,7 @@
       <c r="E130" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F130" s="7" t="inlineStr">
         <is>
           <t>2021.webp</t>
         </is>
@@ -5138,7 +5155,7 @@
       <c r="E131" s="8" t="n">
         <v>1044.23</v>
       </c>
-      <c r="F131" t="inlineStr">
+      <c r="F131" s="7" t="inlineStr">
         <is>
           <t>2708.webp</t>
         </is>
@@ -5171,7 +5188,7 @@
       <c r="E132" s="8" t="n">
         <v>1874.29</v>
       </c>
-      <c r="F132" t="inlineStr">
+      <c r="F132" s="7" t="inlineStr">
         <is>
           <t>3209.webp</t>
         </is>
@@ -5204,7 +5221,7 @@
       <c r="E133" s="8" t="n">
         <v>9750.18</v>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F133" s="7" t="inlineStr">
         <is>
           <t>1163.webp</t>
         </is>
@@ -5237,7 +5254,7 @@
       <c r="E134" s="8" t="n">
         <v>11289.3</v>
       </c>
-      <c r="F134" t="inlineStr">
+      <c r="F134" s="7" t="inlineStr">
         <is>
           <t>1051.webp</t>
         </is>
@@ -5270,7 +5287,7 @@
       <c r="E135" s="8" t="n">
         <v>496.1</v>
       </c>
-      <c r="F135" t="inlineStr">
+      <c r="F135" s="7" t="inlineStr">
         <is>
           <t>107.webp</t>
         </is>
@@ -5303,7 +5320,7 @@
       <c r="E136" s="8" t="n">
         <v>11113.85</v>
       </c>
-      <c r="F136" t="inlineStr">
+      <c r="F136" s="7" t="inlineStr">
         <is>
           <t>882.webp</t>
         </is>
@@ -5336,7 +5353,7 @@
       <c r="E137" s="8" t="n">
         <v>5203</v>
       </c>
-      <c r="F137" t="inlineStr">
+      <c r="F137" s="7" t="inlineStr">
         <is>
           <t>889.webp</t>
         </is>
@@ -5369,7 +5386,7 @@
       <c r="E138" s="8" t="n">
         <v>8808.799999999999</v>
       </c>
-      <c r="F138" t="inlineStr">
+      <c r="F138" s="7" t="inlineStr">
         <is>
           <t>890.webp</t>
         </is>
@@ -5402,7 +5419,7 @@
       <c r="E139" s="8" t="n">
         <v>9388.389999999999</v>
       </c>
-      <c r="F139" t="inlineStr">
+      <c r="F139" s="7" t="inlineStr">
         <is>
           <t>390.webp</t>
         </is>
@@ -5435,7 +5452,7 @@
       <c r="E140" s="8" t="n">
         <v>6521.9</v>
       </c>
-      <c r="F140" t="inlineStr">
+      <c r="F140" s="7" t="inlineStr">
         <is>
           <t>666.webp</t>
         </is>
@@ -5445,7 +5462,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H140" s="14" t="n">
+      <c r="H140" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -5471,7 +5488,7 @@
       <c r="E141" s="8" t="n">
         <v>930.49</v>
       </c>
-      <c r="F141" t="inlineStr">
+      <c r="F141" s="7" t="inlineStr">
         <is>
           <t>667.webp</t>
         </is>
@@ -5504,7 +5521,7 @@
       <c r="E142" s="8" t="n">
         <v>8995.139999999999</v>
       </c>
-      <c r="F142" t="inlineStr">
+      <c r="F142" s="7" t="inlineStr">
         <is>
           <t>798.webp</t>
         </is>
@@ -5537,7 +5554,7 @@
       <c r="E143" s="8" t="n">
         <v>6988</v>
       </c>
-      <c r="F143" t="inlineStr">
+      <c r="F143" s="7" t="inlineStr">
         <is>
           <t>828.webp</t>
         </is>
@@ -5570,7 +5587,7 @@
       <c r="E144" s="8" t="n">
         <v>6982.91</v>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F144" s="7" t="inlineStr">
         <is>
           <t>1024.webp</t>
         </is>
@@ -5603,7 +5620,7 @@
       <c r="E145" s="8" t="n">
         <v>7502</v>
       </c>
-      <c r="F145" t="inlineStr">
+      <c r="F145" s="7" t="inlineStr">
         <is>
           <t>1166.webp</t>
         </is>
@@ -5636,7 +5653,7 @@
       <c r="E146" s="8" t="n">
         <v>5903.59</v>
       </c>
-      <c r="F146" t="inlineStr">
+      <c r="F146" s="7" t="inlineStr">
         <is>
           <t>1169.webp</t>
         </is>
@@ -5669,7 +5686,7 @@
       <c r="E147" s="8" t="n">
         <v>5724.51</v>
       </c>
-      <c r="F147" t="inlineStr">
+      <c r="F147" s="7" t="inlineStr">
         <is>
           <t>687.webp</t>
         </is>
@@ -5702,7 +5719,7 @@
       <c r="E148" s="8" t="n">
         <v>5724.51</v>
       </c>
-      <c r="F148" t="inlineStr">
+      <c r="F148" s="7" t="inlineStr">
         <is>
           <t>8725.webp</t>
         </is>
@@ -5735,7 +5752,7 @@
       <c r="E149" s="8" t="n">
         <v>5833.41</v>
       </c>
-      <c r="F149" t="inlineStr">
+      <c r="F149" s="7" t="inlineStr">
         <is>
           <t>3068.webp</t>
         </is>
@@ -5768,7 +5785,7 @@
       <c r="E150" s="8" t="n">
         <v>5603.51</v>
       </c>
-      <c r="F150" t="inlineStr">
+      <c r="F150" s="7" t="inlineStr">
         <is>
           <t>8713.webp</t>
         </is>
@@ -5778,7 +5795,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H150" s="14" t="n">
+      <c r="H150" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -5804,7 +5821,7 @@
       <c r="E151" s="8" t="n">
         <v>7723.43</v>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F151" s="7" t="inlineStr">
         <is>
           <t>2253.webp</t>
         </is>
@@ -5837,7 +5854,7 @@
       <c r="E152" s="8" t="n">
         <v>5724.51</v>
       </c>
-      <c r="F152" t="inlineStr">
+      <c r="F152" s="7" t="inlineStr">
         <is>
           <t>686.webp</t>
         </is>
@@ -5870,7 +5887,7 @@
       <c r="E153" s="8" t="n">
         <v>7723.43</v>
       </c>
-      <c r="F153" t="inlineStr">
+      <c r="F153" s="7" t="inlineStr">
         <is>
           <t>2900.webp</t>
         </is>
@@ -5903,7 +5920,7 @@
       <c r="E154" s="8" t="n">
         <v>9052.01</v>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="7" t="inlineStr">
         <is>
           <t>1388.webp</t>
         </is>
@@ -5936,7 +5953,7 @@
       <c r="E155" s="8" t="n">
         <v>5315.53</v>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="7" t="inlineStr">
         <is>
           <t>1745.webp</t>
         </is>
@@ -5969,7 +5986,7 @@
       <c r="E156" s="8" t="n">
         <v>6759.06</v>
       </c>
-      <c r="F156" t="inlineStr">
+      <c r="F156" s="7" t="inlineStr">
         <is>
           <t>26.webp</t>
         </is>
@@ -6002,7 +6019,7 @@
       <c r="E157" s="8" t="n">
         <v>1125.3</v>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" s="7" t="inlineStr">
         <is>
           <t>1871.webp</t>
         </is>
@@ -6035,7 +6052,7 @@
       <c r="E158" s="8" t="n">
         <v>6571.51</v>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F158" s="7" t="inlineStr">
         <is>
           <t>1873.webp</t>
         </is>
@@ -6068,7 +6085,7 @@
       <c r="E159" s="8" t="n">
         <v>12463</v>
       </c>
-      <c r="F159" t="inlineStr">
+      <c r="F159" s="7" t="inlineStr">
         <is>
           <t>1996.webp</t>
         </is>
@@ -6078,7 +6095,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H159" s="14" t="n">
+      <c r="H159" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -6104,7 +6121,7 @@
       <c r="E160" s="8" t="n">
         <v>3107.28</v>
       </c>
-      <c r="F160" t="inlineStr">
+      <c r="F160" s="7" t="inlineStr">
         <is>
           <t>1267.webp</t>
         </is>
@@ -6137,7 +6154,7 @@
       <c r="E161" s="8" t="n">
         <v>3977.27</v>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F161" s="7" t="inlineStr">
         <is>
           <t>1234.webp</t>
         </is>
@@ -6170,7 +6187,7 @@
       <c r="E162" s="8" t="n">
         <v>6271.43</v>
       </c>
-      <c r="F162" t="inlineStr">
+      <c r="F162" s="7" t="inlineStr">
         <is>
           <t>2184.webp</t>
         </is>
@@ -6203,7 +6220,7 @@
       <c r="E163" s="8" t="n">
         <v>3891.36</v>
       </c>
-      <c r="F163" t="inlineStr">
+      <c r="F163" s="7" t="inlineStr">
         <is>
           <t>3290.webp</t>
         </is>
@@ -6236,7 +6253,7 @@
       <c r="E164" s="8" t="n">
         <v>3335.97</v>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F164" s="7" t="inlineStr">
         <is>
           <t>7.webp</t>
         </is>
@@ -6269,7 +6286,7 @@
       <c r="E165" s="8" t="n">
         <v>1177.33</v>
       </c>
-      <c r="F165" t="inlineStr">
+      <c r="F165" s="7" t="inlineStr">
         <is>
           <t>35.webp</t>
         </is>
@@ -6302,7 +6319,7 @@
       <c r="E166" s="8" t="n">
         <v>968</v>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="F166" s="7" t="inlineStr">
         <is>
           <t>2590.webp</t>
         </is>
@@ -6335,7 +6352,7 @@
       <c r="E167" s="8" t="n">
         <v>732.05</v>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F167" s="7" t="inlineStr">
         <is>
           <t>3017.webp</t>
         </is>
@@ -6368,7 +6385,7 @@
       <c r="E168" s="8" t="n">
         <v>1551.22</v>
       </c>
-      <c r="F168" t="inlineStr">
+      <c r="F168" s="7" t="inlineStr">
         <is>
           <t>101.webp</t>
         </is>
@@ -6401,7 +6418,7 @@
       <c r="E169" s="8" t="n">
         <v>4129.73</v>
       </c>
-      <c r="F169" t="inlineStr">
+      <c r="F169" s="7" t="inlineStr">
         <is>
           <t>232.webp</t>
         </is>
@@ -6434,7 +6451,7 @@
       <c r="E170" s="8" t="n">
         <v>4129.73</v>
       </c>
-      <c r="F170" t="inlineStr">
+      <c r="F170" s="7" t="inlineStr">
         <is>
           <t>233.webp</t>
         </is>
@@ -6467,7 +6484,7 @@
       <c r="E171" s="8" t="n">
         <v>4662.13</v>
       </c>
-      <c r="F171" t="inlineStr">
+      <c r="F171" s="7" t="inlineStr">
         <is>
           <t>235.webp</t>
         </is>
@@ -6500,7 +6517,7 @@
       <c r="E172" s="8" t="n">
         <v>4829.11</v>
       </c>
-      <c r="F172" t="inlineStr">
+      <c r="F172" s="7" t="inlineStr">
         <is>
           <t>244.webp</t>
         </is>
@@ -6533,7 +6550,7 @@
       <c r="E173" s="8" t="n">
         <v>2885.85</v>
       </c>
-      <c r="F173" t="inlineStr">
+      <c r="F173" s="7" t="inlineStr">
         <is>
           <t>9838.webp</t>
         </is>
@@ -6566,7 +6583,7 @@
       <c r="E174" s="8" t="n">
         <v>2761.22</v>
       </c>
-      <c r="F174" t="inlineStr">
+      <c r="F174" s="7" t="inlineStr">
         <is>
           <t>237.webp</t>
         </is>
@@ -6599,7 +6616,7 @@
       <c r="E175" s="8" t="n">
         <v>5083.21</v>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F175" s="7" t="inlineStr">
         <is>
           <t>238.webp</t>
         </is>
@@ -6632,7 +6649,7 @@
       <c r="E176" s="8" t="n">
         <v>5165.49</v>
       </c>
-      <c r="F176" t="inlineStr">
+      <c r="F176" s="7" t="inlineStr">
         <is>
           <t>9839.webp</t>
         </is>
@@ -6665,7 +6682,7 @@
       <c r="E177" s="8" t="n">
         <v>3698.97</v>
       </c>
-      <c r="F177" t="inlineStr">
+      <c r="F177" s="7" t="inlineStr">
         <is>
           <t>9842.webp</t>
         </is>
@@ -6698,7 +6715,7 @@
       <c r="E178" s="8" t="n">
         <v>2911.26</v>
       </c>
-      <c r="F178" t="inlineStr">
+      <c r="F178" s="7" t="inlineStr">
         <is>
           <t>9840.webp</t>
         </is>
@@ -6731,7 +6748,7 @@
       <c r="E179" s="8" t="n">
         <v>5095.31</v>
       </c>
-      <c r="F179" t="inlineStr">
+      <c r="F179" s="7" t="inlineStr">
         <is>
           <t>261.webp</t>
         </is>
@@ -6764,7 +6781,7 @@
       <c r="E180" s="8" t="n">
         <v>3087.92</v>
       </c>
-      <c r="F180" t="inlineStr">
+      <c r="F180" s="7" t="inlineStr">
         <is>
           <t>9841.webp</t>
         </is>
@@ -6797,7 +6814,7 @@
       <c r="E181" s="8" t="n">
         <v>3477.54</v>
       </c>
-      <c r="F181" t="inlineStr">
+      <c r="F181" s="7" t="inlineStr">
         <is>
           <t>6071.webp</t>
         </is>
@@ -6828,9 +6845,9 @@
         </is>
       </c>
       <c r="E182" s="8" t="n">
-        <v>2420</v>
-      </c>
-      <c r="F182" t="inlineStr">
+        <v>2456.3</v>
+      </c>
+      <c r="F182" s="7" t="inlineStr">
         <is>
           <t>3308.webp</t>
         </is>
@@ -6839,6 +6856,9 @@
         <is>
           <t>Si</t>
         </is>
+      </c>
+      <c r="H182" s="10" t="n">
+        <v>46230.65951186343</v>
       </c>
     </row>
     <row r="183">
@@ -6863,7 +6883,7 @@
       <c r="E183" s="8" t="n">
         <v>3630</v>
       </c>
-      <c r="F183" t="inlineStr">
+      <c r="F183" s="7" t="inlineStr">
         <is>
           <t>3307.webp</t>
         </is>
@@ -6896,7 +6916,7 @@
       <c r="E184" s="8" t="n">
         <v>1367.3</v>
       </c>
-      <c r="F184" t="inlineStr">
+      <c r="F184" s="7" t="inlineStr">
         <is>
           <t>9848.webp</t>
         </is>
@@ -6929,7 +6949,7 @@
       <c r="E185" s="8" t="n">
         <v>960.74</v>
       </c>
-      <c r="F185" t="inlineStr">
+      <c r="F185" s="7" t="inlineStr">
         <is>
           <t>2287.webp</t>
         </is>
@@ -6962,7 +6982,7 @@
       <c r="E186" s="8" t="n">
         <v>1101.1</v>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F186" s="7" t="inlineStr">
         <is>
           <t>839.webp</t>
         </is>
@@ -6995,7 +7015,7 @@
       <c r="E187" s="8" t="n">
         <v>1575.42</v>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="F187" s="7" t="inlineStr">
         <is>
           <t>81.webp</t>
         </is>
@@ -7028,7 +7048,7 @@
       <c r="E188" s="8" t="n">
         <v>1583.89</v>
       </c>
-      <c r="F188" t="inlineStr">
+      <c r="F188" s="7" t="inlineStr">
         <is>
           <t>9851.webp</t>
         </is>
@@ -7061,7 +7081,7 @@
       <c r="E189" s="8" t="n">
         <v>794.97</v>
       </c>
-      <c r="F189" t="inlineStr">
+      <c r="F189" s="7" t="inlineStr">
         <is>
           <t>2937.webp</t>
         </is>
@@ -7094,7 +7114,7 @@
       <c r="E190" s="8" t="n">
         <v>1185.8</v>
       </c>
-      <c r="F190" t="inlineStr">
+      <c r="F190" s="7" t="inlineStr">
         <is>
           <t>3386.webp</t>
         </is>
@@ -7127,7 +7147,7 @@
       <c r="E191" s="8" t="n">
         <v>1137.4</v>
       </c>
-      <c r="F191" t="inlineStr">
+      <c r="F191" s="7" t="inlineStr">
         <is>
           <t>2990.webp</t>
         </is>
@@ -7160,7 +7180,7 @@
       <c r="E192" s="8" t="n">
         <v>660.66</v>
       </c>
-      <c r="F192" t="inlineStr">
+      <c r="F192" s="7" t="inlineStr">
         <is>
           <t>1148.webp</t>
         </is>
@@ -7193,7 +7213,7 @@
       <c r="E193" s="8" t="n">
         <v>1869.45</v>
       </c>
-      <c r="F193" t="inlineStr">
+      <c r="F193" s="7" t="inlineStr">
         <is>
           <t>2945.webp</t>
         </is>
@@ -7226,7 +7246,7 @@
       <c r="E194" s="8" t="n">
         <v>804.65</v>
       </c>
-      <c r="F194" t="inlineStr">
+      <c r="F194" s="7" t="inlineStr">
         <is>
           <t>1641.webp</t>
         </is>
@@ -7259,7 +7279,7 @@
       <c r="E195" s="8" t="n">
         <v>14795.88</v>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F195" s="7" t="inlineStr">
         <is>
           <t>1648.webp</t>
         </is>
@@ -7292,7 +7312,7 @@
       <c r="E196" s="8" t="n">
         <v>792.55</v>
       </c>
-      <c r="F196" t="inlineStr">
+      <c r="F196" s="7" t="inlineStr">
         <is>
           <t>3150.webp</t>
         </is>
@@ -7302,7 +7322,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H196" s="14" t="n">
+      <c r="H196" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -7328,7 +7348,7 @@
       <c r="E197" s="8" t="n">
         <v>1110.78</v>
       </c>
-      <c r="F197" t="inlineStr">
+      <c r="F197" s="7" t="inlineStr">
         <is>
           <t>9850.webp</t>
         </is>
@@ -7361,7 +7381,7 @@
       <c r="E198" s="8" t="n">
         <v>1210</v>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="F198" s="7" t="inlineStr">
         <is>
           <t>8802.webp</t>
         </is>
@@ -7394,7 +7414,7 @@
       <c r="E199" s="8" t="n">
         <v>726</v>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F199" s="7" t="inlineStr">
         <is>
           <t>1797.webp</t>
         </is>
@@ -7427,7 +7447,7 @@
       <c r="E200" s="8" t="n">
         <v>1609.3</v>
       </c>
-      <c r="F200" t="inlineStr">
+      <c r="F200" s="7" t="inlineStr">
         <is>
           <t>3180.webp</t>
         </is>
@@ -7460,7 +7480,7 @@
       <c r="E201" s="8" t="n">
         <v>1409.65</v>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" s="7" t="inlineStr">
         <is>
           <t>1914.webp</t>
         </is>
@@ -7493,7 +7513,7 @@
       <c r="E202" s="8" t="n">
         <v>1616.56</v>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" s="7" t="inlineStr">
         <is>
           <t>3400.webp</t>
         </is>
@@ -7526,7 +7546,7 @@
       <c r="E203" s="8" t="n">
         <v>597.74</v>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="F203" s="7" t="inlineStr">
         <is>
           <t>8797.webp</t>
         </is>
@@ -7559,7 +7579,7 @@
       <c r="E204" s="8" t="n">
         <v>1331</v>
       </c>
-      <c r="F204" t="inlineStr">
+      <c r="F204" s="7" t="inlineStr">
         <is>
           <t>1984.webp</t>
         </is>
@@ -7592,7 +7612,7 @@
       <c r="E205" s="8" t="n">
         <v>1138.61</v>
       </c>
-      <c r="F205" t="inlineStr">
+      <c r="F205" s="7" t="inlineStr">
         <is>
           <t>1991.webp</t>
         </is>
@@ -7625,7 +7645,7 @@
       <c r="E206" s="8" t="n">
         <v>1905.75</v>
       </c>
-      <c r="F206" t="inlineStr">
+      <c r="F206" s="7" t="inlineStr">
         <is>
           <t>2142.webp</t>
         </is>
@@ -7658,7 +7678,7 @@
       <c r="E207" s="8" t="n">
         <v>1897.28</v>
       </c>
-      <c r="F207" t="inlineStr">
+      <c r="F207" s="7" t="inlineStr">
         <is>
           <t>2141.webp</t>
         </is>
@@ -7691,7 +7711,7 @@
       <c r="E208" s="8" t="n">
         <v>1770.23</v>
       </c>
-      <c r="F208" t="inlineStr">
+      <c r="F208" s="7" t="inlineStr">
         <is>
           <t>2633.webp</t>
         </is>
@@ -7724,7 +7744,7 @@
       <c r="E209" s="8" t="n">
         <v>1493.14</v>
       </c>
-      <c r="F209" t="inlineStr">
+      <c r="F209" s="7" t="inlineStr">
         <is>
           <t>2140.webp</t>
         </is>
@@ -7757,7 +7777,7 @@
       <c r="E210" s="8" t="n">
         <v>1432.64</v>
       </c>
-      <c r="F210" t="inlineStr">
+      <c r="F210" s="7" t="inlineStr">
         <is>
           <t>942.webp</t>
         </is>
@@ -7790,7 +7810,7 @@
       <c r="E211" s="8" t="n">
         <v>2299</v>
       </c>
-      <c r="F211" t="inlineStr">
+      <c r="F211" s="7" t="inlineStr">
         <is>
           <t>2809.webp</t>
         </is>
@@ -7823,7 +7843,7 @@
       <c r="E212" s="8" t="n">
         <v>1724.25</v>
       </c>
-      <c r="F212" t="inlineStr">
+      <c r="F212" s="7" t="inlineStr">
         <is>
           <t>8793.webp</t>
         </is>
@@ -7856,7 +7876,7 @@
       <c r="E213" s="8" t="n">
         <v>1839.2</v>
       </c>
-      <c r="F213" t="inlineStr">
+      <c r="F213" s="7" t="inlineStr">
         <is>
           <t>2147.webp</t>
         </is>
@@ -7889,7 +7909,7 @@
       <c r="E214" s="8" t="n">
         <v>1891.23</v>
       </c>
-      <c r="F214" t="inlineStr">
+      <c r="F214" s="7" t="inlineStr">
         <is>
           <t>2149.webp</t>
         </is>
@@ -7922,7 +7942,7 @@
       <c r="E215" s="8" t="n">
         <v>1005.51</v>
       </c>
-      <c r="F215" t="inlineStr">
+      <c r="F215" s="7" t="inlineStr">
         <is>
           <t>19.webp</t>
         </is>
@@ -7955,7 +7975,7 @@
       <c r="E216" s="8" t="n">
         <v>643.72</v>
       </c>
-      <c r="F216" t="inlineStr">
+      <c r="F216" s="7" t="inlineStr">
         <is>
           <t>20.webp</t>
         </is>
@@ -7988,7 +8008,7 @@
       <c r="E217" s="8" t="n">
         <v>2099.35</v>
       </c>
-      <c r="F217" t="inlineStr">
+      <c r="F217" s="7" t="inlineStr">
         <is>
           <t>8800.webp</t>
         </is>
@@ -8021,7 +8041,7 @@
       <c r="E218" s="8" t="n">
         <v>1996.5</v>
       </c>
-      <c r="F218" t="inlineStr">
+      <c r="F218" s="7" t="inlineStr">
         <is>
           <t>8801.webp</t>
         </is>
@@ -8054,7 +8074,7 @@
       <c r="E219" s="8" t="n">
         <v>1357.62</v>
       </c>
-      <c r="F219" t="inlineStr">
+      <c r="F219" s="7" t="inlineStr">
         <is>
           <t>1863.webp</t>
         </is>
@@ -8087,7 +8107,7 @@
       <c r="E220" s="8" t="n">
         <v>2217.93</v>
       </c>
-      <c r="F220" t="inlineStr">
+      <c r="F220" s="7" t="inlineStr">
         <is>
           <t>2662.webp</t>
         </is>
@@ -8120,7 +8140,7 @@
       <c r="E221" s="8" t="n">
         <v>1197.9</v>
       </c>
-      <c r="F221" t="inlineStr">
+      <c r="F221" s="7" t="inlineStr">
         <is>
           <t>156.webp</t>
         </is>
@@ -8153,7 +8173,7 @@
       <c r="E222" s="8" t="n">
         <v>1674.64</v>
       </c>
-      <c r="F222" t="inlineStr">
+      <c r="F222" s="7" t="inlineStr">
         <is>
           <t>302.webp</t>
         </is>
@@ -8186,7 +8206,7 @@
       <c r="E223" s="8" t="n">
         <v>1413.28</v>
       </c>
-      <c r="F223" t="inlineStr">
+      <c r="F223" s="7" t="inlineStr">
         <is>
           <t>373.webp</t>
         </is>
@@ -8219,7 +8239,7 @@
       <c r="E224" s="8" t="n">
         <v>1413.28</v>
       </c>
-      <c r="F224" t="inlineStr">
+      <c r="F224" s="7" t="inlineStr">
         <is>
           <t>8715.webp</t>
         </is>
@@ -8252,7 +8272,7 @@
       <c r="E225" s="8" t="n">
         <v>1073.27</v>
       </c>
-      <c r="F225" t="inlineStr">
+      <c r="F225" s="7" t="inlineStr">
         <is>
           <t>534.webp</t>
         </is>
@@ -8285,7 +8305,7 @@
       <c r="E226" s="8" t="n">
         <v>1739.98</v>
       </c>
-      <c r="F226" t="inlineStr">
+      <c r="F226" s="7" t="inlineStr">
         <is>
           <t>303.webp</t>
         </is>
@@ -8318,7 +8338,7 @@
       <c r="E227" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F227" t="inlineStr">
+      <c r="F227" s="7" t="inlineStr">
         <is>
           <t>705.webp</t>
         </is>
@@ -8328,7 +8348,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H227" s="14" t="n">
+      <c r="H227" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -8354,7 +8374,7 @@
       <c r="E228" s="8" t="n">
         <v>1512.5</v>
       </c>
-      <c r="F228" t="inlineStr">
+      <c r="F228" s="7" t="inlineStr">
         <is>
           <t>1155.webp</t>
         </is>
@@ -8387,7 +8407,7 @@
       <c r="E229" s="8" t="n">
         <v>942.59</v>
       </c>
-      <c r="F229" t="inlineStr">
+      <c r="F229" s="7" t="inlineStr">
         <is>
           <t>1352.webp</t>
         </is>
@@ -8420,7 +8440,7 @@
       <c r="E230" s="8" t="n">
         <v>648.5599999999999</v>
       </c>
-      <c r="F230" t="inlineStr">
+      <c r="F230" s="7" t="inlineStr">
         <is>
           <t>1351.webp</t>
         </is>
@@ -8453,7 +8473,7 @@
       <c r="E231" s="8" t="n">
         <v>1149.5</v>
       </c>
-      <c r="F231" t="inlineStr">
+      <c r="F231" s="7" t="inlineStr">
         <is>
           <t>1764.webp</t>
         </is>
@@ -8463,7 +8483,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H231" s="14" t="n">
+      <c r="H231" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -8489,7 +8509,7 @@
       <c r="E232" s="8" t="n">
         <v>1159.18</v>
       </c>
-      <c r="F232" t="inlineStr">
+      <c r="F232" s="7" t="inlineStr">
         <is>
           <t>1851.webp</t>
         </is>
@@ -8522,7 +8542,7 @@
       <c r="E233" s="8" t="n">
         <v>2184.05</v>
       </c>
-      <c r="F233" t="inlineStr">
+      <c r="F233" s="7" t="inlineStr">
         <is>
           <t>3177.webp</t>
         </is>
@@ -8555,7 +8575,7 @@
       <c r="E234" s="8" t="n">
         <v>635.25</v>
       </c>
-      <c r="F234" t="inlineStr">
+      <c r="F234" s="7" t="inlineStr">
         <is>
           <t>2032.webp</t>
         </is>
@@ -8588,7 +8608,7 @@
       <c r="E235" s="8" t="n">
         <v>1754.5</v>
       </c>
-      <c r="F235" t="inlineStr">
+      <c r="F235" s="7" t="inlineStr">
         <is>
           <t>2033.webp</t>
         </is>
@@ -8621,7 +8641,7 @@
       <c r="E236" s="8" t="n">
         <v>1006.72</v>
       </c>
-      <c r="F236" t="inlineStr">
+      <c r="F236" s="7" t="inlineStr">
         <is>
           <t>8708.webp</t>
         </is>
@@ -8654,7 +8674,7 @@
       <c r="E237" s="8" t="n">
         <v>1641.97</v>
       </c>
-      <c r="F237" t="inlineStr">
+      <c r="F237" s="7" t="inlineStr">
         <is>
           <t>2914.webp</t>
         </is>
@@ -8687,7 +8707,7 @@
       <c r="E238" s="8" t="n">
         <v>2462.35</v>
       </c>
-      <c r="F238" t="inlineStr">
+      <c r="F238" s="7" t="inlineStr">
         <is>
           <t>2913.webp</t>
         </is>
@@ -8720,7 +8740,7 @@
       <c r="E239" s="8" t="n">
         <v>2873.75</v>
       </c>
-      <c r="F239" t="inlineStr">
+      <c r="F239" s="7" t="inlineStr">
         <is>
           <t>3000.webp</t>
         </is>
@@ -8753,7 +8773,7 @@
       <c r="E240" s="8" t="n">
         <v>1006.72</v>
       </c>
-      <c r="F240" t="inlineStr">
+      <c r="F240" s="7" t="inlineStr">
         <is>
           <t>8729.webp</t>
         </is>
@@ -8786,7 +8806,7 @@
       <c r="E241" s="8" t="n">
         <v>4418.92</v>
       </c>
-      <c r="F241" t="inlineStr">
+      <c r="F241" s="7" t="inlineStr">
         <is>
           <t>3093.webp</t>
         </is>
@@ -8819,7 +8839,7 @@
       <c r="E242" s="8" t="n">
         <v>1177.33</v>
       </c>
-      <c r="F242" t="inlineStr">
+      <c r="F242" s="7" t="inlineStr">
         <is>
           <t>3059.webp</t>
         </is>
@@ -8852,7 +8872,7 @@
       <c r="E243" s="8" t="n">
         <v>1201.53</v>
       </c>
-      <c r="F243" t="inlineStr">
+      <c r="F243" s="7" t="inlineStr">
         <is>
           <t>3058.webp</t>
         </is>
@@ -8885,7 +8905,7 @@
       <c r="E244" s="8" t="n">
         <v>1723.04</v>
       </c>
-      <c r="F244" t="inlineStr">
+      <c r="F244" s="7" t="inlineStr">
         <is>
           <t>1498.webp</t>
         </is>
@@ -8918,7 +8938,7 @@
       <c r="E245" s="8" t="n">
         <v>2544.63</v>
       </c>
-      <c r="F245" t="inlineStr">
+      <c r="F245" s="7" t="inlineStr">
         <is>
           <t>1501.webp</t>
         </is>
@@ -8951,7 +8971,7 @@
       <c r="E246" s="8" t="n">
         <v>2956.03</v>
       </c>
-      <c r="F246" t="inlineStr">
+      <c r="F246" s="7" t="inlineStr">
         <is>
           <t>2063.webp</t>
         </is>
@@ -8984,7 +9004,7 @@
       <c r="E247" s="8" t="n">
         <v>1393.92</v>
       </c>
-      <c r="F247" t="inlineStr">
+      <c r="F247" s="7" t="inlineStr">
         <is>
           <t>3140.webp</t>
         </is>
@@ -9017,7 +9037,7 @@
       <c r="E248" s="8" t="n">
         <v>1147.08</v>
       </c>
-      <c r="F248" t="inlineStr">
+      <c r="F248" s="7" t="inlineStr">
         <is>
           <t>3062.webp</t>
         </is>
@@ -9050,7 +9070,7 @@
       <c r="E249" s="8" t="n">
         <v>1460.47</v>
       </c>
-      <c r="F249" t="inlineStr">
+      <c r="F249" s="7" t="inlineStr">
         <is>
           <t>3095.webp</t>
         </is>
@@ -9060,7 +9080,7 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="H249" s="14" t="n">
+      <c r="H249" s="10" t="n">
         <v>46226.47538918981</v>
       </c>
     </row>
@@ -9086,7 +9106,7 @@
       <c r="E250" s="8" t="n">
         <v>2504.7</v>
       </c>
-      <c r="F250" t="inlineStr">
+      <c r="F250" s="7" t="inlineStr">
         <is>
           <t>56.webp</t>
         </is>
@@ -9119,7 +9139,7 @@
       <c r="E251" s="8" t="n">
         <v>1225.73</v>
       </c>
-      <c r="F251" t="inlineStr">
+      <c r="F251" s="7" t="inlineStr">
         <is>
           <t>32.webp</t>
         </is>
@@ -9152,7 +9172,7 @@
       <c r="E252" s="8" t="n">
         <v>1225.73</v>
       </c>
-      <c r="F252" t="inlineStr">
+      <c r="F252" s="7" t="inlineStr">
         <is>
           <t>49.webp</t>
         </is>
@@ -9185,7 +9205,7 @@
       <c r="E253" s="8" t="n">
         <v>1393.92</v>
       </c>
-      <c r="F253" t="inlineStr">
+      <c r="F253" s="7" t="inlineStr">
         <is>
           <t>3098.webp</t>
         </is>
@@ -9218,7 +9238,7 @@
       <c r="E254" s="8" t="n">
         <v>1052.7</v>
       </c>
-      <c r="F254" t="inlineStr">
+      <c r="F254" s="7" t="inlineStr">
         <is>
           <t>368.webp</t>
         </is>
@@ -9251,7 +9271,7 @@
       <c r="E255" s="8" t="n">
         <v>669.13</v>
       </c>
-      <c r="F255" t="inlineStr">
+      <c r="F255" s="7" t="inlineStr">
         <is>
           <t>657.webp</t>
         </is>
@@ -9284,7 +9304,7 @@
       <c r="E256" s="8" t="n">
         <v>871.2</v>
       </c>
-      <c r="F256" t="inlineStr">
+      <c r="F256" s="7" t="inlineStr">
         <is>
           <t>649.webp</t>
         </is>
@@ -9297,11 +9317,11 @@
     </row>
     <row r="257">
       <c r="A257" s="6" t="n">
-        <v>39</v>
+        <v>9858</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ALFAJOR CAP DEL ESPACIO *40G</t>
+          <t>ALFAJOR CAPITÁN DEL ESPACIO X 40G</t>
         </is>
       </c>
       <c r="C257" s="7" t="inlineStr">
@@ -9315,9 +9335,9 @@
         </is>
       </c>
       <c r="E257" s="8" t="n">
-        <v>980.1</v>
-      </c>
-      <c r="F257" t="inlineStr">
+        <v>1355.2</v>
+      </c>
+      <c r="F257" s="7" t="inlineStr">
         <is>
           <t>39.webp</t>
         </is>
@@ -9350,7 +9370,7 @@
       <c r="E258" s="8" t="n">
         <v>4598</v>
       </c>
-      <c r="F258" t="inlineStr">
+      <c r="F258" s="7" t="inlineStr">
         <is>
           <t>3300.webp</t>
         </is>
@@ -9383,7 +9403,7 @@
       <c r="E259" s="8" t="n">
         <v>7146.26</v>
       </c>
-      <c r="F259" t="inlineStr">
+      <c r="F259" s="7" t="inlineStr">
         <is>
           <t>3309.webp</t>
         </is>
@@ -9416,7 +9436,7 @@
       <c r="E260" s="8" t="n">
         <v>7526.2</v>
       </c>
-      <c r="F260" t="inlineStr">
+      <c r="F260" s="7" t="inlineStr">
         <is>
           <t>9859.webp</t>
         </is>
@@ -9449,7 +9469,7 @@
       <c r="E261" s="8" t="n">
         <v>1524.6</v>
       </c>
-      <c r="F261" t="inlineStr">
+      <c r="F261" s="7" t="inlineStr">
         <is>
           <t>9861.webp</t>
         </is>
@@ -9482,7 +9502,7 @@
       <c r="E262" s="8" t="n">
         <v>753.83</v>
       </c>
-      <c r="F262" s="13" t="inlineStr">
+      <c r="F262" s="9" t="inlineStr">
         <is>
           <t>25.webp</t>
         </is>
@@ -9515,7 +9535,7 @@
       <c r="E263" s="8" t="n">
         <v>1234.2</v>
       </c>
-      <c r="F263" s="13" t="inlineStr">
+      <c r="F263" s="9" t="inlineStr">
         <is>
           <t>3401.webp</t>
         </is>
@@ -9548,7 +9568,7 @@
       <c r="E264" s="8" t="n">
         <v>5069.9</v>
       </c>
-      <c r="F264" s="13" t="inlineStr">
+      <c r="F264" s="9" t="inlineStr">
         <is>
           <t>8710.webp</t>
         </is>
@@ -9581,7 +9601,7 @@
       <c r="E265" s="8" t="n">
         <v>4426.18</v>
       </c>
-      <c r="F265" s="13" t="inlineStr">
+      <c r="F265" s="9" t="inlineStr">
         <is>
           <t>3403.webp</t>
         </is>
@@ -9614,7 +9634,7 @@
       <c r="E266" s="8" t="n">
         <v>1401.18</v>
       </c>
-      <c r="F266" s="13" t="inlineStr">
+      <c r="F266" s="9" t="inlineStr">
         <is>
           <t>3269.webp</t>
         </is>
@@ -9647,7 +9667,7 @@
       <c r="E267" s="8" t="n">
         <v>1007.93</v>
       </c>
-      <c r="F267" s="13" t="inlineStr">
+      <c r="F267" s="9" t="inlineStr">
         <is>
           <t>9849.webp</t>
         </is>
@@ -9680,7 +9700,7 @@
       <c r="E268" s="8" t="n">
         <v>1401.18</v>
       </c>
-      <c r="F268" s="13" t="inlineStr">
+      <c r="F268" s="9" t="inlineStr">
         <is>
           <t>427.webp</t>
         </is>
@@ -9713,7 +9733,7 @@
       <c r="E269" s="8" t="n">
         <v>873.62</v>
       </c>
-      <c r="F269" s="13" t="inlineStr">
+      <c r="F269" s="9" t="inlineStr">
         <is>
           <t>435.webp</t>
         </is>
@@ -9746,7 +9766,7 @@
       <c r="E270" s="8" t="n">
         <v>866.36</v>
       </c>
-      <c r="F270" s="13" t="inlineStr">
+      <c r="F270" s="9" t="inlineStr">
         <is>
           <t>437.webp</t>
         </is>
@@ -9779,7 +9799,7 @@
       <c r="E271" s="8" t="n">
         <v>865.15</v>
       </c>
-      <c r="F271" s="13" t="inlineStr">
+      <c r="F271" s="9" t="inlineStr">
         <is>
           <t>2694.webp</t>
         </is>
@@ -9812,7 +9832,7 @@
       <c r="E272" s="8" t="n">
         <v>807.0700000000001</v>
       </c>
-      <c r="F272" s="13" t="inlineStr">
+      <c r="F272" s="9" t="inlineStr">
         <is>
           <t>440.webp</t>
         </is>
@@ -9845,7 +9865,7 @@
       <c r="E273" s="8" t="n">
         <v>744.15</v>
       </c>
-      <c r="F273" s="13" t="inlineStr">
+      <c r="F273" s="9" t="inlineStr">
         <is>
           <t>3402.webp</t>
         </is>
@@ -9878,7 +9898,7 @@
       <c r="E274" s="8" t="n">
         <v>2495.02</v>
       </c>
-      <c r="F274" s="13" t="inlineStr">
+      <c r="F274" s="9" t="inlineStr">
         <is>
           <t>8900.webp</t>
         </is>
@@ -9911,7 +9931,7 @@
       <c r="E275" s="8" t="n">
         <v>2580.93</v>
       </c>
-      <c r="F275" s="13" t="inlineStr">
+      <c r="F275" s="9" t="inlineStr">
         <is>
           <t>3385.webp</t>
         </is>
@@ -9944,7 +9964,7 @@
       <c r="E276" s="8" t="n">
         <v>998.25</v>
       </c>
-      <c r="F276" s="13" t="inlineStr">
+      <c r="F276" s="9" t="inlineStr">
         <is>
           <t>9847.webp</t>
         </is>
@@ -9977,7 +9997,7 @@
       <c r="E277" s="8" t="n">
         <v>3859.9</v>
       </c>
-      <c r="F277" s="13" t="inlineStr">
+      <c r="F277" s="9" t="inlineStr">
         <is>
           <t>8711.webp</t>
         </is>
@@ -10010,7 +10030,7 @@
       <c r="E278" s="8" t="n">
         <v>1128.93</v>
       </c>
-      <c r="F278" s="13" t="inlineStr">
+      <c r="F278" s="9" t="inlineStr">
         <is>
           <t>3266.webp</t>
         </is>
@@ -10043,7 +10063,7 @@
       <c r="E279" s="8" t="n">
         <v>665.5</v>
       </c>
-      <c r="F279" s="13" t="inlineStr">
+      <c r="F279" s="9" t="inlineStr">
         <is>
           <t>3144.webp</t>
         </is>
@@ -10076,7 +10096,7 @@
       <c r="E280" s="8" t="n">
         <v>431.97</v>
       </c>
-      <c r="F280" s="13" t="inlineStr">
+      <c r="F280" s="9" t="inlineStr">
         <is>
           <t>3265.webp</t>
         </is>
@@ -10109,7 +10129,7 @@
       <c r="E281" s="8" t="n">
         <v>2495.02</v>
       </c>
-      <c r="F281" s="13" t="inlineStr">
+      <c r="F281" s="9" t="inlineStr">
         <is>
           <t>1180.webp</t>
         </is>
@@ -10142,7 +10162,7 @@
       <c r="E282" s="8" t="n">
         <v>788.92</v>
       </c>
-      <c r="F282" s="13" t="inlineStr">
+      <c r="F282" s="9" t="inlineStr">
         <is>
           <t>3267.webp</t>
         </is>
@@ -10175,7 +10195,7 @@
       <c r="E283" s="8" t="n">
         <v>1155.55</v>
       </c>
-      <c r="F283" s="13" t="inlineStr">
+      <c r="F283" s="9" t="inlineStr">
         <is>
           <t>1357.webp</t>
         </is>
@@ -10208,7 +10228,7 @@
       <c r="E284" s="8" t="n">
         <v>1473.78</v>
       </c>
-      <c r="F284" s="13" t="inlineStr">
+      <c r="F284" s="9" t="inlineStr">
         <is>
           <t>8809.webp</t>
         </is>
@@ -10241,7 +10261,7 @@
       <c r="E285" s="8" t="n">
         <v>847</v>
       </c>
-      <c r="F285" t="inlineStr">
+      <c r="F285" s="7" t="inlineStr">
         <is>
           <t>sin-imagen.png</t>
         </is>
@@ -10274,7 +10294,7 @@
       <c r="E286" s="8" t="n">
         <v>1339.47</v>
       </c>
-      <c r="F286" s="13" t="inlineStr">
+      <c r="F286" s="9" t="inlineStr">
         <is>
           <t>1508.webp</t>
         </is>
@@ -10307,7 +10327,7 @@
       <c r="E287" s="8" t="n">
         <v>735.6799999999999</v>
       </c>
-      <c r="F287" s="13" t="inlineStr">
+      <c r="F287" s="9" t="inlineStr">
         <is>
           <t>1531.webp</t>
         </is>
@@ -10340,7 +10360,7 @@
       <c r="E288" s="8" t="n">
         <v>1543.96</v>
       </c>
-      <c r="F288" s="13" t="inlineStr">
+      <c r="F288" s="9" t="inlineStr">
         <is>
           <t>1532.webp</t>
         </is>
@@ -10373,7 +10393,7 @@
       <c r="E289" s="8" t="n">
         <v>1125.3</v>
       </c>
-      <c r="F289" s="13" t="inlineStr">
+      <c r="F289" s="9" t="inlineStr">
         <is>
           <t>2426.webp</t>
         </is>
@@ -10406,7 +10426,7 @@
       <c r="E290" s="8" t="n">
         <v>769.5599999999999</v>
       </c>
-      <c r="F290" s="13" t="inlineStr">
+      <c r="F290" s="9" t="inlineStr">
         <is>
           <t>2840.webp</t>
         </is>
@@ -10439,7 +10459,7 @@
       <c r="E291" s="8" t="n">
         <v>1372.14</v>
       </c>
-      <c r="F291" s="13" t="inlineStr">
+      <c r="F291" s="9" t="inlineStr">
         <is>
           <t>8726.webp</t>
         </is>
@@ -10472,7 +10492,7 @@
       <c r="E292" s="8" t="n">
         <v>1066.01</v>
       </c>
-      <c r="F292" s="13" t="inlineStr">
+      <c r="F292" s="9" t="inlineStr">
         <is>
           <t>1631.webp</t>
         </is>
@@ -10505,7 +10525,7 @@
       <c r="E293" s="8" t="n">
         <v>1836.78</v>
       </c>
-      <c r="F293" s="13" t="inlineStr">
+      <c r="F293" s="9" t="inlineStr">
         <is>
           <t>3157.webp</t>
         </is>
@@ -10538,7 +10558,7 @@
       <c r="E294" s="8" t="n">
         <v>1165.23</v>
       </c>
-      <c r="F294" s="13" t="inlineStr">
+      <c r="F294" s="9" t="inlineStr">
         <is>
           <t>8820.webp</t>
         </is>
@@ -10571,12 +10591,144 @@
       <c r="E295" s="8" t="n">
         <v>1040.6</v>
       </c>
-      <c r="F295" s="13" t="inlineStr">
+      <c r="F295" s="9" t="inlineStr">
         <is>
           <t>8709.webp</t>
         </is>
       </c>
       <c r="G295" s="9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="6" t="n">
+        <v>1181</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MERMELADA NOEL LIGHT X 390 GR </t>
+        </is>
+      </c>
+      <c r="C296" s="7" t="inlineStr">
+        <is>
+          <t>Noel</t>
+        </is>
+      </c>
+      <c r="D296" s="7" t="inlineStr">
+        <is>
+          <t>Almacén</t>
+        </is>
+      </c>
+      <c r="E296" s="8" t="n">
+        <v>1950.52</v>
+      </c>
+      <c r="F296" s="9" t="inlineStr">
+        <is>
+          <t>1181.webp</t>
+        </is>
+      </c>
+      <c r="G296" s="9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="6" t="n">
+        <v>8823</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALFAJOR BARRIGON 100 GR     </t>
+        </is>
+      </c>
+      <c r="C297" s="7" t="inlineStr">
+        <is>
+          <t>Barrigón</t>
+        </is>
+      </c>
+      <c r="D297" s="7" t="inlineStr">
+        <is>
+          <t>Alfajores</t>
+        </is>
+      </c>
+      <c r="E297" s="8" t="n">
+        <v>1551.22</v>
+      </c>
+      <c r="F297" s="9" t="inlineStr">
+        <is>
+          <t>8823.webp</t>
+        </is>
+      </c>
+      <c r="G297" s="9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="6" t="n">
+        <v>8890</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALFAJOR BARRIGON 45 GR      </t>
+        </is>
+      </c>
+      <c r="C298" s="7" t="inlineStr">
+        <is>
+          <t>Barrigón</t>
+        </is>
+      </c>
+      <c r="D298" s="7" t="inlineStr">
+        <is>
+          <t>Alfajores</t>
+        </is>
+      </c>
+      <c r="E298" s="8" t="n">
+        <v>424.71</v>
+      </c>
+      <c r="F298" s="9" t="inlineStr">
+        <is>
+          <t>8890.webp</t>
+        </is>
+      </c>
+      <c r="G298" s="9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="6" t="n">
+        <v>8824</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALFAJOR BARRIGON 70 GR      </t>
+        </is>
+      </c>
+      <c r="C299" s="7" t="inlineStr">
+        <is>
+          <t>Barrigón</t>
+        </is>
+      </c>
+      <c r="D299" s="7" t="inlineStr">
+        <is>
+          <t>Alfajores</t>
+        </is>
+      </c>
+      <c r="E299" s="8" t="n">
+        <v>1074.48</v>
+      </c>
+      <c r="F299" s="9" t="inlineStr">
+        <is>
+          <t>8824.webp</t>
+        </is>
+      </c>
+      <c r="G299" s="9" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
@@ -10607,7 +10759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B92"/>
+  <dimension ref="A1:B93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="13.26953125" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -10929,7 +11081,7 @@
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Guaymallén</t>
         </is>
       </c>
     </row>
@@ -11329,6 +11481,13 @@
       <c r="B92" t="inlineStr">
         <is>
           <t>Dánica</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Barrigón</t>
         </is>
       </c>
     </row>

</xml_diff>